<commit_message>
Worked on excel files
Worked on both the physical architecture and the architecture interfaces excel sheets. The interfaces sheet format has been set up but still needs to be filled out with what systems and subsystems interface with what.
</commit_message>
<xml_diff>
--- a/BOBSAT-1/Physical architecture interfaces.xlsx
+++ b/BOBSAT-1/Physical architecture interfaces.xlsx
@@ -1,26 +1,255 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c778b4911c4cd68e/Documents/GitHub/AIAA-Systems-Engineering-Workshop/BOBSAT-1/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="217" documentId="11_F25DC773A252ABDACC104897411C64EE5ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEA9113B-492F-4F26-9256-4FC928BE0BFC}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="10600" yWindow="0" windowWidth="15140" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="69">
+  <si>
+    <t>BOBSAT-1</t>
+  </si>
+  <si>
+    <t>EPS</t>
+  </si>
+  <si>
+    <t>Solar array</t>
+  </si>
+  <si>
+    <t>Power distribution</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>ADCS</t>
+  </si>
+  <si>
+    <t>1.2.1</t>
+  </si>
+  <si>
+    <t>1.2.2</t>
+  </si>
+  <si>
+    <t>1.1.1</t>
+  </si>
+  <si>
+    <t>1.1.1.1</t>
+  </si>
+  <si>
+    <t>1.1.2</t>
+  </si>
+  <si>
+    <t>Power generation</t>
+  </si>
+  <si>
+    <t>wiring</t>
+  </si>
+  <si>
+    <t>Sensors</t>
+  </si>
+  <si>
+    <t>Sun sensor</t>
+  </si>
+  <si>
+    <t>Star tracker</t>
+  </si>
+  <si>
+    <t>Magnotometer</t>
+  </si>
+  <si>
+    <t>Gyroscope</t>
+  </si>
+  <si>
+    <t>Actuators</t>
+  </si>
+  <si>
+    <t>Magno torquers</t>
+  </si>
+  <si>
+    <t>Reaction wheels</t>
+  </si>
+  <si>
+    <t>S&amp;E</t>
+  </si>
+  <si>
+    <t>Structural integrity</t>
+  </si>
+  <si>
+    <t>Chassis</t>
+  </si>
+  <si>
+    <t>buss assembly</t>
+  </si>
+  <si>
+    <t>Thermal management</t>
+  </si>
+  <si>
+    <t>Multi layer insulaiton</t>
+  </si>
+  <si>
+    <t>heat radiators</t>
+  </si>
+  <si>
+    <t>heaters</t>
+  </si>
+  <si>
+    <t>radiation shielding</t>
+  </si>
+  <si>
+    <t>Payload</t>
+  </si>
+  <si>
+    <t>hyperspecral imager</t>
+  </si>
+  <si>
+    <t>hyperscape x50</t>
+  </si>
+  <si>
+    <t>Communications</t>
+  </si>
+  <si>
+    <t>Uplink and downlink antenna</t>
+  </si>
+  <si>
+    <t>Radio</t>
+  </si>
+  <si>
+    <t>C&amp;DH</t>
+  </si>
+  <si>
+    <t>Onboard Computer</t>
+  </si>
+  <si>
+    <t>Ground</t>
+  </si>
+  <si>
+    <t>Ground computer</t>
+  </si>
+  <si>
+    <t>ground antennas</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Mechanical interfaces Diagram</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>1.1.2.1</t>
+  </si>
+  <si>
+    <t>1.1.2.2</t>
+  </si>
+  <si>
+    <t>1.2.1.1</t>
+  </si>
+  <si>
+    <t>1.2.1.2</t>
+  </si>
+  <si>
+    <t>1.2.1.3</t>
+  </si>
+  <si>
+    <t>1.2.1.4</t>
+  </si>
+  <si>
+    <t>1.2.2.1</t>
+  </si>
+  <si>
+    <t>1.2.2.2</t>
+  </si>
+  <si>
+    <t>1.3.1</t>
+  </si>
+  <si>
+    <t>1.3.1.1</t>
+  </si>
+  <si>
+    <t>1.3.1.2</t>
+  </si>
+  <si>
+    <t>1.3.2</t>
+  </si>
+  <si>
+    <t>1.3.2.1</t>
+  </si>
+  <si>
+    <t>1.3.2.2</t>
+  </si>
+  <si>
+    <t>1.3.2.3</t>
+  </si>
+  <si>
+    <t>1.3.2.4</t>
+  </si>
+  <si>
+    <t>1.4.1</t>
+  </si>
+  <si>
+    <t>1.4.1.2</t>
+  </si>
+  <si>
+    <t>1.5.1</t>
+  </si>
+  <si>
+    <t>1.5.2</t>
+  </si>
+  <si>
+    <t>1.6.1</t>
+  </si>
+  <si>
+    <t>1.7.1</t>
+  </si>
+  <si>
+    <t>1.7.2</t>
+  </si>
+  <si>
+    <t>Ground antennas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       X</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +257,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +300,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +589,772 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AQ47"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.54296875" style="1" customWidth="1"/>
+    <col min="2" max="39" width="8.7265625" style="1"/>
+    <col min="40" max="40" width="3.453125" style="1" customWidth="1"/>
+    <col min="41" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+    </row>
+    <row r="2" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC2" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AF2" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AI2" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="AK2" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="AL2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>2</v>
+      </c>
+      <c r="AO2" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="AP2" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
+      <c r="AC3" s="4"/>
+      <c r="AD3" s="4"/>
+      <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="4"/>
+      <c r="AI3" s="4"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="4"/>
+      <c r="AL3" s="4"/>
+      <c r="AM3" s="4"/>
+      <c r="AN3" s="4"/>
+      <c r="AO3" s="4"/>
+      <c r="AP3" s="4"/>
+      <c r="AQ3" s="4"/>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="4"/>
+      <c r="AB4" s="4"/>
+      <c r="AC4" s="4"/>
+      <c r="AD4" s="4"/>
+      <c r="AE4" s="4"/>
+      <c r="AF4" s="4"/>
+      <c r="AG4" s="4"/>
+      <c r="AH4" s="4"/>
+      <c r="AI4" s="4"/>
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="4"/>
+      <c r="AL4" s="4"/>
+      <c r="AM4" s="4"/>
+      <c r="AN4" s="4"/>
+      <c r="AO4" s="4"/>
+      <c r="AP4" s="4"/>
+      <c r="AQ4" s="4"/>
+    </row>
+    <row r="5" spans="1:43" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
+      <c r="AE5" s="4"/>
+      <c r="AF5" s="4"/>
+      <c r="AG5" s="4"/>
+      <c r="AH5" s="4"/>
+      <c r="AI5" s="4"/>
+      <c r="AJ5" s="4"/>
+      <c r="AK5" s="4"/>
+      <c r="AL5" s="4"/>
+      <c r="AM5" s="4"/>
+      <c r="AN5" s="4"/>
+      <c r="AO5" s="4"/>
+      <c r="AP5" s="4"/>
+      <c r="AQ5" s="4"/>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="V6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AN6" s="4"/>
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="AN7" s="4"/>
+    </row>
+    <row r="8" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="AN8" s="4"/>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="AN9" s="4"/>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="AN10" s="4"/>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1.2</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="AN11" s="4"/>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="AN12" s="4"/>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="AN13" s="4"/>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="AN14" s="4"/>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="AN15" s="4"/>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="AN16" s="4"/>
+    </row>
+    <row r="17" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="AN17" s="4"/>
+    </row>
+    <row r="18" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="AN18" s="4"/>
+    </row>
+    <row r="19" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="AN19" s="4"/>
+    </row>
+    <row r="20" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="1">
+        <v>1.3</v>
+      </c>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="AN20" s="4"/>
+    </row>
+    <row r="21" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A21" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="AN21" s="4"/>
+    </row>
+    <row r="22" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="AN22" s="4"/>
+    </row>
+    <row r="23" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="AN23" s="4"/>
+    </row>
+    <row r="24" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A24" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="AN24" s="4"/>
+    </row>
+    <row r="25" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="AN25" s="4"/>
+    </row>
+    <row r="26" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="AN26" s="4"/>
+    </row>
+    <row r="27" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="AN27" s="4"/>
+    </row>
+    <row r="28" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="AN28" s="4"/>
+    </row>
+    <row r="29" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A29" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="1">
+        <v>1.4</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="AN29" s="4"/>
+    </row>
+    <row r="30" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A30" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="AN30" s="4"/>
+    </row>
+    <row r="31" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="AN31" s="4"/>
+    </row>
+    <row r="32" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A32" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="AN32" s="4"/>
+    </row>
+    <row r="33" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A33" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="AN33" s="4"/>
+    </row>
+    <row r="34" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A34" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="AN34" s="4"/>
+    </row>
+    <row r="35" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A35" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="1">
+        <v>1.6</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="AN35" s="4"/>
+    </row>
+    <row r="36" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="AN36" s="4"/>
+    </row>
+    <row r="37" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A37" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="AN37" s="4"/>
+    </row>
+    <row r="38" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="AN38" s="4"/>
+    </row>
+    <row r="39" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="AN39" s="4"/>
+    </row>
+    <row r="40" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B40" s="1">
+        <v>2</v>
+      </c>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="4"/>
+      <c r="O40" s="4"/>
+      <c r="P40" s="4"/>
+      <c r="Q40" s="4"/>
+      <c r="R40" s="4"/>
+      <c r="S40" s="4"/>
+      <c r="T40" s="4"/>
+      <c r="U40" s="4"/>
+      <c r="V40" s="4"/>
+      <c r="W40" s="4"/>
+      <c r="X40" s="4"/>
+      <c r="Y40" s="4"/>
+      <c r="Z40" s="4"/>
+      <c r="AA40" s="4"/>
+      <c r="AB40" s="4"/>
+      <c r="AC40" s="4"/>
+      <c r="AD40" s="4"/>
+      <c r="AE40" s="4"/>
+      <c r="AF40" s="4"/>
+      <c r="AG40" s="4"/>
+      <c r="AH40" s="4"/>
+      <c r="AI40" s="4"/>
+      <c r="AJ40" s="4"/>
+      <c r="AK40" s="4"/>
+      <c r="AL40" s="4"/>
+      <c r="AM40" s="4"/>
+      <c r="AN40" s="4"/>
+    </row>
+    <row r="41" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" s="1">
+        <v>2.1</v>
+      </c>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+    </row>
+    <row r="42" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+    </row>
+    <row r="43" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+    </row>
+    <row r="44" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C44"/>
+      <c r="D44"/>
+    </row>
+    <row r="45" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="C45"/>
+      <c r="D45"/>
+    </row>
+    <row r="46" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="C46"/>
+      <c r="D46"/>
+    </row>
+    <row r="47" spans="1:40" x14ac:dyDescent="0.35">
+      <c r="C47"/>
+      <c r="D47"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>